<commit_message>
Swapped 36t pulley for 40t and did center distance calcs
</commit_message>
<xml_diff>
--- a/Analysis/APWCR_Hand_Calculations.xlsx
+++ b/Analysis/APWCR_Hand_Calculations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshu\Documents\UT_Files\Senior_Design_Repos\APWCR_CAD_FILES\Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{428BA473-80E9-447E-BBA3-071BDAFFE00A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70AC07DF-FA75-466B-8F7B-8FB917F5708C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Waste Collection Mechanism" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="97">
   <si>
     <t>Mechanism Properties</t>
   </si>
@@ -326,13 +326,64 @@
   <si>
     <t>Friction Torque</t>
   </si>
+  <si>
+    <t>Belt Drive Dimensioning</t>
+  </si>
+  <si>
+    <t>Pulley 1</t>
+  </si>
+  <si>
+    <t>Pitch</t>
+  </si>
+  <si>
+    <t>Teeth Count</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Pulley 2</t>
+  </si>
+  <si>
+    <t>Belt</t>
+  </si>
+  <si>
+    <t>Number of Teeth</t>
+  </si>
+  <si>
+    <t>Belt Pitch length</t>
+  </si>
+  <si>
+    <t>Outer Diameter</t>
+  </si>
+  <si>
+    <t>Pitch Diameter</t>
+  </si>
+  <si>
+    <t>Linear Belt Span, A</t>
+  </si>
+  <si>
+    <t>Pulley Wrap, P</t>
+  </si>
+  <si>
+    <t>Pulley Diameter Difference Squared, d</t>
+  </si>
+  <si>
+    <t>Quadratic Distance Correction Term, Q</t>
+  </si>
+  <si>
+    <t>Required Center Distance, C</t>
+  </si>
+  <si>
+    <t>mm^2</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -426,7 +477,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -666,6 +717,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -674,7 +740,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -693,78 +759,84 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="2" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" xfId="4" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="20" xfId="3" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -783,12 +855,22 @@
     <xf numFmtId="2" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="3" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="2" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" xfId="4" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="20" xfId="3" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Calculation" xfId="3" builtinId="22"/>
@@ -858,6 +940,139 @@
         </a:extLst>
       </xdr:spPr>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>100013</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>114299</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>210959</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>123824</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8BD68204-D59E-3ECE-7664-CED1F5A2C90F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3857626" y="9115424"/>
+          <a:ext cx="7549971" cy="733425"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>61912</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>428953</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4D7AC66-20E1-4231-E0C3-AF2E0FB36C9A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3833813" y="8505825"/>
+          <a:ext cx="9087178" cy="695325"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>257173</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>128588</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>442912</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>170813</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{528FB093-6D3E-2C85-68A2-FDDBF9DAA248}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:srcRect l="1750" r="8626" b="8719"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4014786" y="9853613"/>
+          <a:ext cx="6329364" cy="3142613"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1190,11 +1405,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:J44"/>
+  <dimension ref="B1:J70"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="4.53125" customWidth="1"/>
-    <col min="2" max="2" width="30.3984375" customWidth="1"/>
+    <col min="2" max="2" width="33.1328125" customWidth="1"/>
     <col min="3" max="3" width="8.53125" customWidth="1"/>
     <col min="4" max="4" width="6.3984375" customWidth="1"/>
     <col min="5" max="5" width="22.3984375" customWidth="1"/>
@@ -1204,33 +1419,33 @@
   <sheetData>
     <row r="1" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:10" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="21"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="42"/>
     </row>
     <row r="3" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="23"/>
+      <c r="C3" s="44"/>
       <c r="D3" s="8"/>
-      <c r="E3" s="23" t="s">
+      <c r="E3" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="23"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="8"/>
-      <c r="H3" s="23" t="s">
+      <c r="H3" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="23"/>
+      <c r="I3" s="44"/>
       <c r="J3" s="9"/>
     </row>
     <row r="4" spans="2:10" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
@@ -1256,7 +1471,7 @@
       <c r="H4" t="s">
         <v>16</v>
       </c>
-      <c r="I4" s="48">
+      <c r="I4" s="18">
         <f>C6*C11</f>
         <v>328.08950740312991</v>
       </c>
@@ -1278,7 +1493,7 @@
       <c r="E5" t="s">
         <v>79</v>
       </c>
-      <c r="F5" s="48">
+      <c r="F5" s="18">
         <f>F4*C7</f>
         <v>15.8</v>
       </c>
@@ -1288,7 +1503,7 @@
       <c r="H5" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="49">
+      <c r="I5" s="19">
         <f>I4*C10</f>
         <v>213.25817981203446</v>
       </c>
@@ -1300,7 +1515,7 @@
       <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="48">
+      <c r="C6" s="18">
         <f>C5*0.86796165979664</f>
         <v>8.2022376850782486</v>
       </c>
@@ -1358,17 +1573,17 @@
         <v>0.65</v>
       </c>
       <c r="D10" s="11"/>
-      <c r="E10" s="24" t="s">
+      <c r="E10" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="25"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="36">
+      <c r="F10" s="30"/>
+      <c r="G10" s="45"/>
+      <c r="H10" s="33">
         <f>(I5/F6) - 1</f>
         <v>0.79964708702138787</v>
       </c>
-      <c r="I10" s="37"/>
-      <c r="J10" s="38"/>
+      <c r="I10" s="34"/>
+      <c r="J10" s="35"/>
     </row>
     <row r="11" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B11" s="4" t="s">
@@ -1378,42 +1593,42 @@
         <v>40</v>
       </c>
       <c r="D11" s="6"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="29"/>
-      <c r="H11" s="39"/>
-      <c r="I11" s="40"/>
-      <c r="J11" s="41"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="36"/>
+      <c r="I11" s="37"/>
+      <c r="J11" s="38"/>
     </row>
     <row r="14" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="15" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="40" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
-      <c r="J15" s="21"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="41"/>
+      <c r="G15" s="41"/>
+      <c r="H15" s="41"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="42"/>
     </row>
     <row r="16" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="C16" s="23"/>
+      <c r="C16" s="44"/>
       <c r="D16" s="8"/>
-      <c r="E16" s="23" t="s">
+      <c r="E16" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F16" s="23"/>
+      <c r="F16" s="44"/>
       <c r="G16" s="8"/>
-      <c r="H16" s="23" t="s">
+      <c r="H16" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="I16" s="23"/>
+      <c r="I16" s="44"/>
       <c r="J16" s="9"/>
     </row>
     <row r="17" spans="2:10" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
@@ -1429,7 +1644,7 @@
       <c r="E17" t="s">
         <v>73</v>
       </c>
-      <c r="F17" s="48">
+      <c r="F17" s="18">
         <f>C18*C17</f>
         <v>0.75</v>
       </c>
@@ -1439,7 +1654,7 @@
       <c r="H17" t="s">
         <v>16</v>
       </c>
-      <c r="I17" s="48">
+      <c r="I17" s="18">
         <f>C20</f>
         <v>8.6796165979663993</v>
       </c>
@@ -1457,7 +1672,7 @@
       <c r="E18" t="s">
         <v>75</v>
       </c>
-      <c r="F18" s="48">
+      <c r="F18" s="18">
         <f>F17*C21</f>
         <v>0.9375</v>
       </c>
@@ -1467,7 +1682,7 @@
       <c r="H18" t="s">
         <v>17</v>
       </c>
-      <c r="I18" s="49">
+      <c r="I18" s="19">
         <f>I17</f>
         <v>8.6796165979663993</v>
       </c>
@@ -1488,7 +1703,7 @@
       <c r="E19" t="s">
         <v>11</v>
       </c>
-      <c r="F19" s="49">
+      <c r="F19" s="19">
         <f>((F18/COS(RADIANS(C23)))*C24*SIN(RADIANS(C22)))*C25</f>
         <v>1.8194062500000001</v>
       </c>
@@ -1501,7 +1716,7 @@
       <c r="B20" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C20" s="48">
+      <c r="C20" s="18">
         <f>C19*0.86796165979664</f>
         <v>8.6796165979663993</v>
       </c>
@@ -1515,7 +1730,7 @@
       <c r="B21" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C21" s="50">
+      <c r="C21" s="20">
         <v>1.25</v>
       </c>
       <c r="D21" s="11"/>
@@ -1525,7 +1740,7 @@
       <c r="B22" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C22" s="50">
+      <c r="C22" s="20">
         <v>90</v>
       </c>
       <c r="D22" s="11" t="s">
@@ -1537,7 +1752,7 @@
       <c r="B23" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C23" s="50">
+      <c r="C23" s="20">
         <v>0</v>
       </c>
       <c r="D23" s="11" t="s">
@@ -1549,247 +1764,484 @@
       <c r="B24" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C24" s="50">
+      <c r="C24" s="20">
         <v>1.2938000000000001</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="E24" s="24" t="s">
+      <c r="E24" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="F24" s="25"/>
-      <c r="G24" s="26"/>
-      <c r="H24" s="42">
+      <c r="F24" s="30"/>
+      <c r="G24" s="45"/>
+      <c r="H24" s="48">
         <f>(I18/F19) - 1</f>
         <v>3.7705764438076423</v>
       </c>
-      <c r="I24" s="43"/>
-      <c r="J24" s="44"/>
+      <c r="I24" s="49"/>
+      <c r="J24" s="50"/>
     </row>
     <row r="25" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B25" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C25" s="51">
+      <c r="C25" s="21">
         <v>1.5</v>
       </c>
       <c r="D25" s="6"/>
-      <c r="E25" s="27"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="29"/>
-      <c r="H25" s="45"/>
-      <c r="I25" s="46"/>
-      <c r="J25" s="47"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="46"/>
+      <c r="H25" s="51"/>
+      <c r="I25" s="52"/>
+      <c r="J25" s="53"/>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B27" s="18" t="e" vm="1">
+      <c r="B27" s="47" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="18"/>
-      <c r="G27" s="18"/>
-      <c r="H27" s="18"/>
-      <c r="I27" s="18"/>
-      <c r="J27" s="18"/>
+      <c r="C27" s="47"/>
+      <c r="D27" s="47"/>
+      <c r="E27" s="47"/>
+      <c r="F27" s="47"/>
+      <c r="G27" s="47"/>
+      <c r="H27" s="47"/>
+      <c r="I27" s="47"/>
+      <c r="J27" s="47"/>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="18"/>
+      <c r="B28" s="47"/>
+      <c r="C28" s="47"/>
+      <c r="D28" s="47"/>
+      <c r="E28" s="47"/>
+      <c r="F28" s="47"/>
+      <c r="G28" s="47"/>
+      <c r="H28" s="47"/>
+      <c r="I28" s="47"/>
+      <c r="J28" s="47"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="18"/>
-      <c r="G29" s="18"/>
-      <c r="H29" s="18"/>
-      <c r="I29" s="18"/>
-      <c r="J29" s="18"/>
+      <c r="B29" s="47"/>
+      <c r="C29" s="47"/>
+      <c r="D29" s="47"/>
+      <c r="E29" s="47"/>
+      <c r="F29" s="47"/>
+      <c r="G29" s="47"/>
+      <c r="H29" s="47"/>
+      <c r="I29" s="47"/>
+      <c r="J29" s="47"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="18"/>
-      <c r="G30" s="18"/>
-      <c r="H30" s="18"/>
-      <c r="I30" s="18"/>
-      <c r="J30" s="18"/>
+      <c r="B30" s="47"/>
+      <c r="C30" s="47"/>
+      <c r="D30" s="47"/>
+      <c r="E30" s="47"/>
+      <c r="F30" s="47"/>
+      <c r="G30" s="47"/>
+      <c r="H30" s="47"/>
+      <c r="I30" s="47"/>
+      <c r="J30" s="47"/>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="18"/>
-      <c r="F31" s="18"/>
-      <c r="G31" s="18"/>
-      <c r="H31" s="18"/>
-      <c r="I31" s="18"/>
-      <c r="J31" s="18"/>
+      <c r="B31" s="47"/>
+      <c r="C31" s="47"/>
+      <c r="D31" s="47"/>
+      <c r="E31" s="47"/>
+      <c r="F31" s="47"/>
+      <c r="G31" s="47"/>
+      <c r="H31" s="47"/>
+      <c r="I31" s="47"/>
+      <c r="J31" s="47"/>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="18"/>
-      <c r="J32" s="18"/>
+      <c r="B32" s="47"/>
+      <c r="C32" s="47"/>
+      <c r="D32" s="47"/>
+      <c r="E32" s="47"/>
+      <c r="F32" s="47"/>
+      <c r="G32" s="47"/>
+      <c r="H32" s="47"/>
+      <c r="I32" s="47"/>
+      <c r="J32" s="47"/>
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="18"/>
-      <c r="H33" s="18"/>
-      <c r="I33" s="18"/>
-      <c r="J33" s="18"/>
+      <c r="B33" s="47"/>
+      <c r="C33" s="47"/>
+      <c r="D33" s="47"/>
+      <c r="E33" s="47"/>
+      <c r="F33" s="47"/>
+      <c r="G33" s="47"/>
+      <c r="H33" s="47"/>
+      <c r="I33" s="47"/>
+      <c r="J33" s="47"/>
     </row>
     <row r="34" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B34" s="18"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="18"/>
-      <c r="E34" s="18"/>
-      <c r="F34" s="18"/>
-      <c r="G34" s="18"/>
-      <c r="H34" s="18"/>
-      <c r="I34" s="18"/>
-      <c r="J34" s="18"/>
+      <c r="B34" s="47"/>
+      <c r="C34" s="47"/>
+      <c r="D34" s="47"/>
+      <c r="E34" s="47"/>
+      <c r="F34" s="47"/>
+      <c r="G34" s="47"/>
+      <c r="H34" s="47"/>
+      <c r="I34" s="47"/>
+      <c r="J34" s="47"/>
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B35" s="18"/>
-      <c r="C35" s="18"/>
-      <c r="D35" s="18"/>
-      <c r="E35" s="18"/>
-      <c r="F35" s="18"/>
-      <c r="G35" s="18"/>
-      <c r="H35" s="18"/>
-      <c r="I35" s="18"/>
-      <c r="J35" s="18"/>
+      <c r="B35" s="47"/>
+      <c r="C35" s="47"/>
+      <c r="D35" s="47"/>
+      <c r="E35" s="47"/>
+      <c r="F35" s="47"/>
+      <c r="G35" s="47"/>
+      <c r="H35" s="47"/>
+      <c r="I35" s="47"/>
+      <c r="J35" s="47"/>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B36" s="18"/>
-      <c r="C36" s="18"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="18"/>
-      <c r="G36" s="18"/>
-      <c r="H36" s="18"/>
-      <c r="I36" s="18"/>
-      <c r="J36" s="18"/>
+      <c r="B36" s="47"/>
+      <c r="C36" s="47"/>
+      <c r="D36" s="47"/>
+      <c r="E36" s="47"/>
+      <c r="F36" s="47"/>
+      <c r="G36" s="47"/>
+      <c r="H36" s="47"/>
+      <c r="I36" s="47"/>
+      <c r="J36" s="47"/>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B37" s="18"/>
-      <c r="C37" s="18"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="18"/>
-      <c r="F37" s="18"/>
-      <c r="G37" s="18"/>
-      <c r="H37" s="18"/>
-      <c r="I37" s="18"/>
-      <c r="J37" s="18"/>
+      <c r="B37" s="47"/>
+      <c r="C37" s="47"/>
+      <c r="D37" s="47"/>
+      <c r="E37" s="47"/>
+      <c r="F37" s="47"/>
+      <c r="G37" s="47"/>
+      <c r="H37" s="47"/>
+      <c r="I37" s="47"/>
+      <c r="J37" s="47"/>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B38" s="18"/>
-      <c r="C38" s="18"/>
-      <c r="D38" s="18"/>
-      <c r="E38" s="18"/>
-      <c r="F38" s="18"/>
-      <c r="G38" s="18"/>
-      <c r="H38" s="18"/>
-      <c r="I38" s="18"/>
-      <c r="J38" s="18"/>
+      <c r="B38" s="47"/>
+      <c r="C38" s="47"/>
+      <c r="D38" s="47"/>
+      <c r="E38" s="47"/>
+      <c r="F38" s="47"/>
+      <c r="G38" s="47"/>
+      <c r="H38" s="47"/>
+      <c r="I38" s="47"/>
+      <c r="J38" s="47"/>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B39" s="18"/>
-      <c r="C39" s="18"/>
-      <c r="D39" s="18"/>
-      <c r="E39" s="18"/>
-      <c r="F39" s="18"/>
-      <c r="G39" s="18"/>
-      <c r="H39" s="18"/>
-      <c r="I39" s="18"/>
-      <c r="J39" s="18"/>
+      <c r="B39" s="47"/>
+      <c r="C39" s="47"/>
+      <c r="D39" s="47"/>
+      <c r="E39" s="47"/>
+      <c r="F39" s="47"/>
+      <c r="G39" s="47"/>
+      <c r="H39" s="47"/>
+      <c r="I39" s="47"/>
+      <c r="J39" s="47"/>
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B40" s="18"/>
-      <c r="C40" s="18"/>
-      <c r="D40" s="18"/>
-      <c r="E40" s="18"/>
-      <c r="F40" s="18"/>
-      <c r="G40" s="18"/>
-      <c r="H40" s="18"/>
-      <c r="I40" s="18"/>
-      <c r="J40" s="18"/>
+      <c r="B40" s="47"/>
+      <c r="C40" s="47"/>
+      <c r="D40" s="47"/>
+      <c r="E40" s="47"/>
+      <c r="F40" s="47"/>
+      <c r="G40" s="47"/>
+      <c r="H40" s="47"/>
+      <c r="I40" s="47"/>
+      <c r="J40" s="47"/>
     </row>
     <row r="41" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B41" s="18"/>
-      <c r="C41" s="18"/>
-      <c r="D41" s="18"/>
-      <c r="E41" s="18"/>
-      <c r="F41" s="18"/>
-      <c r="G41" s="18"/>
-      <c r="H41" s="18"/>
-      <c r="I41" s="18"/>
-      <c r="J41" s="18"/>
+      <c r="B41" s="47"/>
+      <c r="C41" s="47"/>
+      <c r="D41" s="47"/>
+      <c r="E41" s="47"/>
+      <c r="F41" s="47"/>
+      <c r="G41" s="47"/>
+      <c r="H41" s="47"/>
+      <c r="I41" s="47"/>
+      <c r="J41" s="47"/>
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B42" s="18"/>
-      <c r="C42" s="18"/>
-      <c r="D42" s="18"/>
-      <c r="E42" s="18"/>
-      <c r="F42" s="18"/>
-      <c r="G42" s="18"/>
-      <c r="H42" s="18"/>
-      <c r="I42" s="18"/>
-      <c r="J42" s="18"/>
+      <c r="B42" s="47"/>
+      <c r="C42" s="47"/>
+      <c r="D42" s="47"/>
+      <c r="E42" s="47"/>
+      <c r="F42" s="47"/>
+      <c r="G42" s="47"/>
+      <c r="H42" s="47"/>
+      <c r="I42" s="47"/>
+      <c r="J42" s="47"/>
     </row>
     <row r="43" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B43" s="18"/>
-      <c r="C43" s="18"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="18"/>
-      <c r="F43" s="18"/>
-      <c r="G43" s="18"/>
-      <c r="H43" s="18"/>
-      <c r="I43" s="18"/>
-      <c r="J43" s="18"/>
+      <c r="B43" s="47"/>
+      <c r="C43" s="47"/>
+      <c r="D43" s="47"/>
+      <c r="E43" s="47"/>
+      <c r="F43" s="47"/>
+      <c r="G43" s="47"/>
+      <c r="H43" s="47"/>
+      <c r="I43" s="47"/>
+      <c r="J43" s="47"/>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B44" s="18"/>
-      <c r="C44" s="18"/>
-      <c r="D44" s="18"/>
-      <c r="E44" s="18"/>
-      <c r="F44" s="18"/>
-      <c r="G44" s="18"/>
-      <c r="H44" s="18"/>
-      <c r="I44" s="18"/>
-      <c r="J44" s="18"/>
+      <c r="B44" s="47"/>
+      <c r="C44" s="47"/>
+      <c r="D44" s="47"/>
+      <c r="E44" s="47"/>
+      <c r="F44" s="47"/>
+      <c r="G44" s="47"/>
+      <c r="H44" s="47"/>
+      <c r="I44" s="47"/>
+      <c r="J44" s="47"/>
+    </row>
+    <row r="47" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="48" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B48" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="C48" s="27"/>
+      <c r="D48" s="28"/>
+      <c r="E48" s="57"/>
+      <c r="F48" s="57"/>
+      <c r="G48" s="57"/>
+      <c r="H48" s="57"/>
+      <c r="I48" s="57"/>
+      <c r="J48" s="57"/>
+    </row>
+    <row r="49" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B49" s="54" t="s">
+        <v>81</v>
+      </c>
+      <c r="C49" s="55"/>
+      <c r="D49" s="56"/>
+    </row>
+    <row r="50" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B50" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C50" s="58">
+        <v>2</v>
+      </c>
+      <c r="D50" s="15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="51" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B51" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C51" s="58">
+        <v>18</v>
+      </c>
+      <c r="D51" s="15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="52" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B52" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C52" s="58">
+        <v>16.13</v>
+      </c>
+      <c r="D52" s="15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="53" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B53" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C53" s="58">
+        <v>11.46</v>
+      </c>
+      <c r="D53" s="15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="54" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B54" s="2"/>
+      <c r="C54" s="59"/>
+      <c r="D54" s="1"/>
+    </row>
+    <row r="55" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B55" s="54" t="s">
+        <v>85</v>
+      </c>
+      <c r="C55" s="55"/>
+      <c r="D55" s="56"/>
+    </row>
+    <row r="56" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B56" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C56" s="58">
+        <v>2</v>
+      </c>
+      <c r="D56" s="15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="57" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B57" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C57" s="58">
+        <v>40</v>
+      </c>
+      <c r="D57" s="15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="58" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B58" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C58" s="58">
+        <v>30.73</v>
+      </c>
+      <c r="D58" s="15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="59" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B59" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C59" s="58">
+        <v>25.48</v>
+      </c>
+      <c r="D59" s="15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="60" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B60" s="2"/>
+      <c r="C60" s="59"/>
+      <c r="D60" s="1"/>
+    </row>
+    <row r="61" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B61" s="54" t="s">
+        <v>86</v>
+      </c>
+      <c r="C61" s="55"/>
+      <c r="D61" s="56"/>
+    </row>
+    <row r="62" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B62" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C62" s="58">
+        <v>2</v>
+      </c>
+      <c r="D62" s="15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="63" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B63" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C63" s="58">
+        <v>228</v>
+      </c>
+      <c r="D63" s="15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="64" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B64" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C64" s="60">
+        <f>C62*C63</f>
+        <v>456</v>
+      </c>
+      <c r="D64" s="15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="65" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B65" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C65" s="60">
+        <f>(PI()/2)*(C53+C59)</f>
+        <v>58.025216311803476</v>
+      </c>
+      <c r="D65" s="61" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="66" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B66" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C66" s="60">
+        <f>C64-C65</f>
+        <v>397.97478368819651</v>
+      </c>
+      <c r="D66" s="61" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="67" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B67" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C67" s="60">
+        <f>(C59-C53)^2</f>
+        <v>196.56039999999999</v>
+      </c>
+      <c r="D67" s="61" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="68" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B68" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C68" s="60">
+        <f>SQRT((C66^2) -(2*C67) )</f>
+        <v>397.48057518785345</v>
+      </c>
+      <c r="D68" s="61" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="69" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B69" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C69" s="60">
+        <f>(C66+C68)/(4)</f>
+        <v>198.8638397190125</v>
+      </c>
+      <c r="D69" s="61" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="70" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B70" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C70" s="62">
+        <f>C69/25.4</f>
+        <v>7.829285028307579</v>
+      </c>
+      <c r="D70" s="63" t="s">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="E10:G11"/>
-    <mergeCell ref="H10:J11"/>
+  <mergeCells count="17">
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B61:D61"/>
     <mergeCell ref="B27:J44"/>
     <mergeCell ref="B15:J15"/>
     <mergeCell ref="B16:C16"/>
@@ -1797,6 +2249,12 @@
     <mergeCell ref="H16:I16"/>
     <mergeCell ref="E24:G25"/>
     <mergeCell ref="H24:J25"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="E10:G11"/>
+    <mergeCell ref="H10:J11"/>
   </mergeCells>
   <conditionalFormatting sqref="H10">
     <cfRule type="colorScale" priority="2">
@@ -1841,33 +2299,33 @@
   <sheetData>
     <row r="1" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
-      <c r="J2" s="34"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="28"/>
     </row>
     <row r="3" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="31"/>
+      <c r="C3" s="25"/>
       <c r="D3" s="8"/>
-      <c r="E3" s="30" t="s">
+      <c r="E3" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="F3" s="31"/>
+      <c r="F3" s="25"/>
       <c r="G3" s="8"/>
-      <c r="H3" s="30" t="s">
+      <c r="H3" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="I3" s="31"/>
+      <c r="I3" s="25"/>
       <c r="J3" s="9"/>
     </row>
     <row r="4" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -1884,7 +2342,7 @@
       <c r="E4" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="53">
+      <c r="F4" s="23">
         <f>C15*SIN(RADIANS(C5))</f>
         <v>2.5051158172811778</v>
       </c>
@@ -1894,7 +2352,7 @@
       <c r="H4" t="s">
         <v>46</v>
       </c>
-      <c r="I4" s="52">
+      <c r="I4" s="22">
         <f>C10</f>
         <v>8.2022376850782486</v>
       </c>
@@ -1915,7 +2373,7 @@
       <c r="E5" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="48">
+      <c r="F5" s="18">
         <f>C13*C15*COS(RADIANS(C5))</f>
         <v>2.6737237856022396</v>
       </c>
@@ -1925,7 +2383,7 @@
       <c r="H5" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="I5" s="49">
+      <c r="I5" s="19">
         <f>C10*C6*C7</f>
         <v>13.943804064633023</v>
       </c>
@@ -1943,7 +2401,7 @@
       <c r="E6" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="48">
+      <c r="F6" s="18">
         <f>(C15/C14)*(C11)</f>
         <v>0.41959346055821478</v>
       </c>
@@ -1962,7 +2420,7 @@
       <c r="E7" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="48">
+      <c r="F7" s="18">
         <f>SUM(F4:F6)</f>
         <v>5.5984330634416324</v>
       </c>
@@ -1984,7 +2442,7 @@
       <c r="E8" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="48">
+      <c r="F8" s="18">
         <f>F7/2</f>
         <v>2.7992165317208162</v>
       </c>
@@ -2007,7 +2465,7 @@
       <c r="E9" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="49">
+      <c r="F9" s="19">
         <f>F8*C4*C12</f>
         <v>9.6572970344368141</v>
       </c>
@@ -2020,7 +2478,7 @@
       <c r="B10" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="48">
+      <c r="C10" s="18">
         <f>C9*0.86796165979664</f>
         <v>8.2022376850782486</v>
       </c>
@@ -2071,17 +2529,17 @@
       <c r="D14" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="24" t="s">
+      <c r="E14" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="36">
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="33">
         <f>(I5/F9) - 1</f>
         <v>0.44386198487123418</v>
       </c>
-      <c r="I14" s="37"/>
-      <c r="J14" s="38"/>
+      <c r="I14" s="34"/>
+      <c r="J14" s="35"/>
     </row>
     <row r="15" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B15" s="4" t="s">
@@ -2093,34 +2551,34 @@
       <c r="D15" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="27"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="39"/>
-      <c r="I15" s="40"/>
-      <c r="J15" s="41"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="32"/>
+      <c r="H15" s="36"/>
+      <c r="I15" s="37"/>
+      <c r="J15" s="38"/>
     </row>
     <row r="16" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="17" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B17" s="32" t="s">
+      <c r="B17" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="33"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="34"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="28"/>
     </row>
     <row r="18" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B18" s="30" t="s">
+      <c r="B18" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="C18" s="31"/>
-      <c r="E18" s="30" t="s">
+      <c r="C18" s="25"/>
+      <c r="E18" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F18" s="35"/>
-      <c r="G18" s="31"/>
+      <c r="F18" s="39"/>
+      <c r="G18" s="25"/>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.45">
       <c r="B19" s="2" t="s">

</xml_diff>

<commit_message>
Adjusted Waste Collection Arm Sizing
</commit_message>
<xml_diff>
--- a/Analysis/APWCR_Hand_Calculations.xlsx
+++ b/Analysis/APWCR_Hand_Calculations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshu\Documents\UT_Files\Senior_Design_Repos\APWCR_CAD_FILES\Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70AC07DF-FA75-466B-8F7B-8FB917F5708C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA4FE2B2-C5B4-4861-B76B-4F850E2694A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -740,7 +740,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -765,112 +765,107 @@
     <xf numFmtId="164" fontId="1" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="18" xfId="4" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="20" xfId="3" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="3" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Calculation" xfId="3" builtinId="22"/>
@@ -1419,33 +1414,33 @@
   <sheetData>
     <row r="1" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:10" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="42"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="35"/>
     </row>
     <row r="3" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="44"/>
+      <c r="C3" s="37"/>
       <c r="D3" s="8"/>
-      <c r="E3" s="44" t="s">
+      <c r="E3" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="44"/>
+      <c r="F3" s="37"/>
       <c r="G3" s="8"/>
-      <c r="H3" s="44" t="s">
+      <c r="H3" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="44"/>
+      <c r="I3" s="37"/>
       <c r="J3" s="9"/>
     </row>
     <row r="4" spans="2:10" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
@@ -1453,7 +1448,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="10">
-        <v>7.9</v>
+        <v>7.83</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>2</v>
@@ -1463,7 +1458,7 @@
       </c>
       <c r="F4" s="3">
         <f>C8*(C4)</f>
-        <v>63.2</v>
+        <v>62.64</v>
       </c>
       <c r="G4" s="11" t="s">
         <v>13</v>
@@ -1495,7 +1490,7 @@
       </c>
       <c r="F5" s="18">
         <f>F4*C7</f>
-        <v>15.8</v>
+        <v>15.66</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>13</v>
@@ -1527,7 +1522,7 @@
       </c>
       <c r="F6" s="12">
         <f>(F4+F5)*C9</f>
-        <v>118.5</v>
+        <v>117.44999999999999</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>13</v>
@@ -1573,17 +1568,17 @@
         <v>0.65</v>
       </c>
       <c r="D10" s="11"/>
-      <c r="E10" s="29" t="s">
+      <c r="E10" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="30"/>
-      <c r="G10" s="45"/>
-      <c r="H10" s="33">
+      <c r="F10" s="39"/>
+      <c r="G10" s="40"/>
+      <c r="H10" s="50">
         <f>(I5/F6) - 1</f>
-        <v>0.79964708702138787</v>
-      </c>
-      <c r="I10" s="34"/>
-      <c r="J10" s="35"/>
+        <v>0.81573588601136215</v>
+      </c>
+      <c r="I10" s="51"/>
+      <c r="J10" s="52"/>
     </row>
     <row r="11" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B11" s="4" t="s">
@@ -1593,42 +1588,42 @@
         <v>40</v>
       </c>
       <c r="D11" s="6"/>
-      <c r="E11" s="31"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="36"/>
-      <c r="I11" s="37"/>
-      <c r="J11" s="38"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="43"/>
+      <c r="H11" s="53"/>
+      <c r="I11" s="54"/>
+      <c r="J11" s="55"/>
     </row>
     <row r="14" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="15" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="41"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="41"/>
-      <c r="F15" s="41"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="41"/>
-      <c r="I15" s="41"/>
-      <c r="J15" s="42"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="34"/>
+      <c r="I15" s="34"/>
+      <c r="J15" s="35"/>
     </row>
     <row r="16" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B16" s="43" t="s">
+      <c r="B16" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="C16" s="44"/>
+      <c r="C16" s="37"/>
       <c r="D16" s="8"/>
-      <c r="E16" s="44" t="s">
+      <c r="E16" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="F16" s="44"/>
+      <c r="F16" s="37"/>
       <c r="G16" s="8"/>
-      <c r="H16" s="44" t="s">
+      <c r="H16" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="I16" s="44"/>
+      <c r="I16" s="37"/>
       <c r="J16" s="9"/>
     </row>
     <row r="17" spans="2:10" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
@@ -1770,17 +1765,17 @@
       <c r="D24" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="E24" s="29" t="s">
+      <c r="E24" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="F24" s="30"/>
-      <c r="G24" s="45"/>
-      <c r="H24" s="48">
+      <c r="F24" s="39"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="44">
         <f>(I18/F19) - 1</f>
         <v>3.7705764438076423</v>
       </c>
-      <c r="I24" s="49"/>
-      <c r="J24" s="50"/>
+      <c r="I24" s="45"/>
+      <c r="J24" s="46"/>
     </row>
     <row r="25" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B25" s="4" t="s">
@@ -1790,212 +1785,212 @@
         <v>1.5</v>
       </c>
       <c r="D25" s="6"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="32"/>
-      <c r="G25" s="46"/>
-      <c r="H25" s="51"/>
-      <c r="I25" s="52"/>
-      <c r="J25" s="53"/>
+      <c r="E25" s="41"/>
+      <c r="F25" s="42"/>
+      <c r="G25" s="43"/>
+      <c r="H25" s="47"/>
+      <c r="I25" s="48"/>
+      <c r="J25" s="49"/>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B27" s="47" t="e" vm="1">
+      <c r="B27" s="32" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C27" s="47"/>
-      <c r="D27" s="47"/>
-      <c r="E27" s="47"/>
-      <c r="F27" s="47"/>
-      <c r="G27" s="47"/>
-      <c r="H27" s="47"/>
-      <c r="I27" s="47"/>
-      <c r="J27" s="47"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B28" s="47"/>
-      <c r="C28" s="47"/>
-      <c r="D28" s="47"/>
-      <c r="E28" s="47"/>
-      <c r="F28" s="47"/>
-      <c r="G28" s="47"/>
-      <c r="H28" s="47"/>
-      <c r="I28" s="47"/>
-      <c r="J28" s="47"/>
+      <c r="B28" s="32"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="32"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B29" s="47"/>
-      <c r="C29" s="47"/>
-      <c r="D29" s="47"/>
-      <c r="E29" s="47"/>
-      <c r="F29" s="47"/>
-      <c r="G29" s="47"/>
-      <c r="H29" s="47"/>
-      <c r="I29" s="47"/>
-      <c r="J29" s="47"/>
+      <c r="B29" s="32"/>
+      <c r="C29" s="32"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="32"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B30" s="47"/>
-      <c r="C30" s="47"/>
-      <c r="D30" s="47"/>
-      <c r="E30" s="47"/>
-      <c r="F30" s="47"/>
-      <c r="G30" s="47"/>
-      <c r="H30" s="47"/>
-      <c r="I30" s="47"/>
-      <c r="J30" s="47"/>
+      <c r="B30" s="32"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="32"/>
+      <c r="I30" s="32"/>
+      <c r="J30" s="32"/>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B31" s="47"/>
-      <c r="C31" s="47"/>
-      <c r="D31" s="47"/>
-      <c r="E31" s="47"/>
-      <c r="F31" s="47"/>
-      <c r="G31" s="47"/>
-      <c r="H31" s="47"/>
-      <c r="I31" s="47"/>
-      <c r="J31" s="47"/>
+      <c r="B31" s="32"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="32"/>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B32" s="47"/>
-      <c r="C32" s="47"/>
-      <c r="D32" s="47"/>
-      <c r="E32" s="47"/>
-      <c r="F32" s="47"/>
-      <c r="G32" s="47"/>
-      <c r="H32" s="47"/>
-      <c r="I32" s="47"/>
-      <c r="J32" s="47"/>
+      <c r="B32" s="32"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="32"/>
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B33" s="47"/>
-      <c r="C33" s="47"/>
-      <c r="D33" s="47"/>
-      <c r="E33" s="47"/>
-      <c r="F33" s="47"/>
-      <c r="G33" s="47"/>
-      <c r="H33" s="47"/>
-      <c r="I33" s="47"/>
-      <c r="J33" s="47"/>
+      <c r="B33" s="32"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="32"/>
     </row>
     <row r="34" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B34" s="47"/>
-      <c r="C34" s="47"/>
-      <c r="D34" s="47"/>
-      <c r="E34" s="47"/>
-      <c r="F34" s="47"/>
-      <c r="G34" s="47"/>
-      <c r="H34" s="47"/>
-      <c r="I34" s="47"/>
-      <c r="J34" s="47"/>
+      <c r="B34" s="32"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="32"/>
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B35" s="47"/>
-      <c r="C35" s="47"/>
-      <c r="D35" s="47"/>
-      <c r="E35" s="47"/>
-      <c r="F35" s="47"/>
-      <c r="G35" s="47"/>
-      <c r="H35" s="47"/>
-      <c r="I35" s="47"/>
-      <c r="J35" s="47"/>
+      <c r="B35" s="32"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="32"/>
+      <c r="H35" s="32"/>
+      <c r="I35" s="32"/>
+      <c r="J35" s="32"/>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B36" s="47"/>
-      <c r="C36" s="47"/>
-      <c r="D36" s="47"/>
-      <c r="E36" s="47"/>
-      <c r="F36" s="47"/>
-      <c r="G36" s="47"/>
-      <c r="H36" s="47"/>
-      <c r="I36" s="47"/>
-      <c r="J36" s="47"/>
+      <c r="B36" s="32"/>
+      <c r="C36" s="32"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="32"/>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B37" s="47"/>
-      <c r="C37" s="47"/>
-      <c r="D37" s="47"/>
-      <c r="E37" s="47"/>
-      <c r="F37" s="47"/>
-      <c r="G37" s="47"/>
-      <c r="H37" s="47"/>
-      <c r="I37" s="47"/>
-      <c r="J37" s="47"/>
+      <c r="B37" s="32"/>
+      <c r="C37" s="32"/>
+      <c r="D37" s="32"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="32"/>
+      <c r="J37" s="32"/>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B38" s="47"/>
-      <c r="C38" s="47"/>
-      <c r="D38" s="47"/>
-      <c r="E38" s="47"/>
-      <c r="F38" s="47"/>
-      <c r="G38" s="47"/>
-      <c r="H38" s="47"/>
-      <c r="I38" s="47"/>
-      <c r="J38" s="47"/>
+      <c r="B38" s="32"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="32"/>
+      <c r="J38" s="32"/>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B39" s="47"/>
-      <c r="C39" s="47"/>
-      <c r="D39" s="47"/>
-      <c r="E39" s="47"/>
-      <c r="F39" s="47"/>
-      <c r="G39" s="47"/>
-      <c r="H39" s="47"/>
-      <c r="I39" s="47"/>
-      <c r="J39" s="47"/>
+      <c r="B39" s="32"/>
+      <c r="C39" s="32"/>
+      <c r="D39" s="32"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="32"/>
+      <c r="J39" s="32"/>
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B40" s="47"/>
-      <c r="C40" s="47"/>
-      <c r="D40" s="47"/>
-      <c r="E40" s="47"/>
-      <c r="F40" s="47"/>
-      <c r="G40" s="47"/>
-      <c r="H40" s="47"/>
-      <c r="I40" s="47"/>
-      <c r="J40" s="47"/>
+      <c r="B40" s="32"/>
+      <c r="C40" s="32"/>
+      <c r="D40" s="32"/>
+      <c r="E40" s="32"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="32"/>
+      <c r="I40" s="32"/>
+      <c r="J40" s="32"/>
     </row>
     <row r="41" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B41" s="47"/>
-      <c r="C41" s="47"/>
-      <c r="D41" s="47"/>
-      <c r="E41" s="47"/>
-      <c r="F41" s="47"/>
-      <c r="G41" s="47"/>
-      <c r="H41" s="47"/>
-      <c r="I41" s="47"/>
-      <c r="J41" s="47"/>
+      <c r="B41" s="32"/>
+      <c r="C41" s="32"/>
+      <c r="D41" s="32"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="32"/>
+      <c r="I41" s="32"/>
+      <c r="J41" s="32"/>
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B42" s="47"/>
-      <c r="C42" s="47"/>
-      <c r="D42" s="47"/>
-      <c r="E42" s="47"/>
-      <c r="F42" s="47"/>
-      <c r="G42" s="47"/>
-      <c r="H42" s="47"/>
-      <c r="I42" s="47"/>
-      <c r="J42" s="47"/>
+      <c r="B42" s="32"/>
+      <c r="C42" s="32"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="32"/>
+      <c r="F42" s="32"/>
+      <c r="G42" s="32"/>
+      <c r="H42" s="32"/>
+      <c r="I42" s="32"/>
+      <c r="J42" s="32"/>
     </row>
     <row r="43" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B43" s="47"/>
-      <c r="C43" s="47"/>
-      <c r="D43" s="47"/>
-      <c r="E43" s="47"/>
-      <c r="F43" s="47"/>
-      <c r="G43" s="47"/>
-      <c r="H43" s="47"/>
-      <c r="I43" s="47"/>
-      <c r="J43" s="47"/>
+      <c r="B43" s="32"/>
+      <c r="C43" s="32"/>
+      <c r="D43" s="32"/>
+      <c r="E43" s="32"/>
+      <c r="F43" s="32"/>
+      <c r="G43" s="32"/>
+      <c r="H43" s="32"/>
+      <c r="I43" s="32"/>
+      <c r="J43" s="32"/>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B44" s="47"/>
-      <c r="C44" s="47"/>
-      <c r="D44" s="47"/>
-      <c r="E44" s="47"/>
-      <c r="F44" s="47"/>
-      <c r="G44" s="47"/>
-      <c r="H44" s="47"/>
-      <c r="I44" s="47"/>
-      <c r="J44" s="47"/>
+      <c r="B44" s="32"/>
+      <c r="C44" s="32"/>
+      <c r="D44" s="32"/>
+      <c r="E44" s="32"/>
+      <c r="F44" s="32"/>
+      <c r="G44" s="32"/>
+      <c r="H44" s="32"/>
+      <c r="I44" s="32"/>
+      <c r="J44" s="32"/>
     </row>
     <row r="47" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="48" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -2004,25 +1999,25 @@
       </c>
       <c r="C48" s="27"/>
       <c r="D48" s="28"/>
-      <c r="E48" s="57"/>
-      <c r="F48" s="57"/>
-      <c r="G48" s="57"/>
-      <c r="H48" s="57"/>
-      <c r="I48" s="57"/>
-      <c r="J48" s="57"/>
+      <c r="E48" s="11"/>
+      <c r="F48" s="11"/>
+      <c r="G48" s="11"/>
+      <c r="H48" s="11"/>
+      <c r="I48" s="11"/>
+      <c r="J48" s="11"/>
     </row>
     <row r="49" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B49" s="54" t="s">
+      <c r="B49" s="29" t="s">
         <v>81</v>
       </c>
-      <c r="C49" s="55"/>
-      <c r="D49" s="56"/>
+      <c r="C49" s="30"/>
+      <c r="D49" s="31"/>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B50" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C50" s="58">
+      <c r="C50" s="10">
         <v>2</v>
       </c>
       <c r="D50" s="15" t="s">
@@ -2033,7 +2028,7 @@
       <c r="B51" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C51" s="58">
+      <c r="C51" s="10">
         <v>18</v>
       </c>
       <c r="D51" s="15" t="s">
@@ -2044,7 +2039,7 @@
       <c r="B52" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C52" s="58">
+      <c r="C52" s="10">
         <v>16.13</v>
       </c>
       <c r="D52" s="15" t="s">
@@ -2055,7 +2050,7 @@
       <c r="B53" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C53" s="58">
+      <c r="C53" s="10">
         <v>11.46</v>
       </c>
       <c r="D53" s="15" t="s">
@@ -2064,21 +2059,20 @@
     </row>
     <row r="54" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B54" s="2"/>
-      <c r="C54" s="59"/>
       <c r="D54" s="1"/>
     </row>
     <row r="55" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B55" s="54" t="s">
+      <c r="B55" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="C55" s="55"/>
-      <c r="D55" s="56"/>
+      <c r="C55" s="30"/>
+      <c r="D55" s="31"/>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B56" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C56" s="58">
+      <c r="C56" s="10">
         <v>2</v>
       </c>
       <c r="D56" s="15" t="s">
@@ -2089,7 +2083,7 @@
       <c r="B57" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C57" s="58">
+      <c r="C57" s="10">
         <v>40</v>
       </c>
       <c r="D57" s="15" t="s">
@@ -2100,7 +2094,7 @@
       <c r="B58" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C58" s="58">
+      <c r="C58" s="10">
         <v>30.73</v>
       </c>
       <c r="D58" s="15" t="s">
@@ -2111,7 +2105,7 @@
       <c r="B59" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C59" s="58">
+      <c r="C59" s="10">
         <v>25.48</v>
       </c>
       <c r="D59" s="15" t="s">
@@ -2120,21 +2114,20 @@
     </row>
     <row r="60" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B60" s="2"/>
-      <c r="C60" s="59"/>
       <c r="D60" s="1"/>
     </row>
     <row r="61" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B61" s="54" t="s">
+      <c r="B61" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="C61" s="55"/>
-      <c r="D61" s="56"/>
+      <c r="C61" s="30"/>
+      <c r="D61" s="31"/>
     </row>
     <row r="62" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B62" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C62" s="58">
+      <c r="C62" s="10">
         <v>2</v>
       </c>
       <c r="D62" s="15" t="s">
@@ -2145,7 +2138,7 @@
       <c r="B63" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C63" s="58">
+      <c r="C63" s="10">
         <v>228</v>
       </c>
       <c r="D63" s="15" t="s">
@@ -2156,7 +2149,7 @@
       <c r="B64" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C64" s="60">
+      <c r="C64" s="3">
         <f>C62*C63</f>
         <v>456</v>
       </c>
@@ -2168,11 +2161,11 @@
       <c r="B65" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C65" s="60">
+      <c r="C65" s="3">
         <f>(PI()/2)*(C53+C59)</f>
         <v>58.025216311803476</v>
       </c>
-      <c r="D65" s="61" t="s">
+      <c r="D65" s="15" t="s">
         <v>50</v>
       </c>
     </row>
@@ -2180,11 +2173,11 @@
       <c r="B66" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C66" s="60">
+      <c r="C66" s="3">
         <f>C64-C65</f>
         <v>397.97478368819651</v>
       </c>
-      <c r="D66" s="61" t="s">
+      <c r="D66" s="15" t="s">
         <v>50</v>
       </c>
     </row>
@@ -2192,11 +2185,11 @@
       <c r="B67" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C67" s="60">
+      <c r="C67" s="3">
         <f>(C59-C53)^2</f>
         <v>196.56039999999999</v>
       </c>
-      <c r="D67" s="61" t="s">
+      <c r="D67" s="15" t="s">
         <v>96</v>
       </c>
     </row>
@@ -2204,11 +2197,11 @@
       <c r="B68" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C68" s="60">
+      <c r="C68" s="3">
         <f>SQRT((C66^2) -(2*C67) )</f>
         <v>397.48057518785345</v>
       </c>
-      <c r="D68" s="61" t="s">
+      <c r="D68" s="15" t="s">
         <v>50</v>
       </c>
     </row>
@@ -2216,11 +2209,11 @@
       <c r="B69" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C69" s="60">
+      <c r="C69" s="3">
         <f>(C66+C68)/(4)</f>
         <v>198.8638397190125</v>
       </c>
-      <c r="D69" s="61" t="s">
+      <c r="D69" s="15" t="s">
         <v>50</v>
       </c>
     </row>
@@ -2228,33 +2221,33 @@
       <c r="B70" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="C70" s="62">
+      <c r="C70" s="24">
         <f>C69/25.4</f>
         <v>7.829285028307579</v>
       </c>
-      <c r="D70" s="63" t="s">
+      <c r="D70" s="25" t="s">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B48:D48"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="B61:D61"/>
-    <mergeCell ref="B27:J44"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="E10:G11"/>
+    <mergeCell ref="H10:J11"/>
     <mergeCell ref="B15:J15"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="H16:I16"/>
     <mergeCell ref="E24:G25"/>
     <mergeCell ref="H24:J25"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="E10:G11"/>
-    <mergeCell ref="H10:J11"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="B27:J44"/>
   </mergeCells>
   <conditionalFormatting sqref="H10">
     <cfRule type="colorScale" priority="2">
@@ -2312,20 +2305,20 @@
       <c r="J2" s="28"/>
     </row>
     <row r="3" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="25"/>
+      <c r="C3" s="57"/>
       <c r="D3" s="8"/>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="F3" s="25"/>
+      <c r="F3" s="57"/>
       <c r="G3" s="8"/>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="56" t="s">
         <v>45</v>
       </c>
-      <c r="I3" s="25"/>
+      <c r="I3" s="57"/>
       <c r="J3" s="9"/>
     </row>
     <row r="4" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -2529,17 +2522,17 @@
       <c r="D14" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="29" t="s">
+      <c r="E14" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="F14" s="30"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="33">
+      <c r="F14" s="39"/>
+      <c r="G14" s="39"/>
+      <c r="H14" s="50">
         <f>(I5/F9) - 1</f>
         <v>0.44386198487123418</v>
       </c>
-      <c r="I14" s="34"/>
-      <c r="J14" s="35"/>
+      <c r="I14" s="51"/>
+      <c r="J14" s="52"/>
     </row>
     <row r="15" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B15" s="4" t="s">
@@ -2551,12 +2544,12 @@
       <c r="D15" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="31"/>
-      <c r="F15" s="32"/>
-      <c r="G15" s="32"/>
-      <c r="H15" s="36"/>
-      <c r="I15" s="37"/>
-      <c r="J15" s="38"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="42"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="53"/>
+      <c r="I15" s="54"/>
+      <c r="J15" s="55"/>
     </row>
     <row r="16" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="17" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -2570,15 +2563,15 @@
       <c r="G17" s="28"/>
     </row>
     <row r="18" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="56" t="s">
         <v>49</v>
       </c>
-      <c r="C18" s="25"/>
-      <c r="E18" s="24" t="s">
+      <c r="C18" s="57"/>
+      <c r="E18" s="56" t="s">
         <v>58</v>
       </c>
-      <c r="F18" s="39"/>
-      <c r="G18" s="25"/>
+      <c r="F18" s="58"/>
+      <c r="G18" s="57"/>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.45">
       <c r="B19" s="2" t="s">

</xml_diff>

<commit_message>
Finished stabilizer Bar Implementation
</commit_message>
<xml_diff>
--- a/Analysis/APWCR_Hand_Calculations.xlsx
+++ b/Analysis/APWCR_Hand_Calculations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshu\Documents\UT_Files\Senior_Design_Repos\APWCR_CAD_FILES\Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA4FE2B2-C5B4-4861-B76B-4F850E2694A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1308E3C-3F5E-49A6-B419-18DA2A40EE23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="113">
   <si>
     <t>Mechanism Properties</t>
   </si>
@@ -377,13 +377,62 @@
   <si>
     <t>mm^2</t>
   </si>
+  <si>
+    <t>Stabilizer Bar Deflection Check</t>
+  </si>
+  <si>
+    <t>Young's Modulus</t>
+  </si>
+  <si>
+    <t>Density</t>
+  </si>
+  <si>
+    <t>psi</t>
+  </si>
+  <si>
+    <t>lb/in^3</t>
+  </si>
+  <si>
+    <t>OD</t>
+  </si>
+  <si>
+    <t>Length</t>
+  </si>
+  <si>
+    <t>Area moment of Inertia</t>
+  </si>
+  <si>
+    <t>in^4</t>
+  </si>
+  <si>
+    <t>Load, P</t>
+  </si>
+  <si>
+    <t>Max deflection</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>Cross-Sectional Area</t>
+  </si>
+  <si>
+    <t>Volume</t>
+  </si>
+  <si>
+    <t>in^2</t>
+  </si>
+  <si>
+    <t>in^3</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.000000"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -477,7 +526,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -732,6 +781,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -740,7 +804,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -768,6 +832,75 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -788,75 +921,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -866,6 +930,16 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Calculation" xfId="3" builtinId="22"/>
@@ -1400,7 +1474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:J70"/>
+  <dimension ref="B1:J84"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="4.53125" customWidth="1"/>
@@ -1414,33 +1488,33 @@
   <sheetData>
     <row r="1" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:10" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="35"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="28"/>
     </row>
     <row r="3" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="37"/>
+      <c r="C3" s="30"/>
       <c r="D3" s="8"/>
-      <c r="E3" s="37" t="s">
+      <c r="E3" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="37"/>
+      <c r="F3" s="30"/>
       <c r="G3" s="8"/>
-      <c r="H3" s="37" t="s">
+      <c r="H3" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="37"/>
+      <c r="I3" s="30"/>
       <c r="J3" s="9"/>
     </row>
     <row r="4" spans="2:10" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
@@ -1458,7 +1532,7 @@
       </c>
       <c r="F4" s="3">
         <f>C8*(C4)</f>
-        <v>62.64</v>
+        <v>70.47</v>
       </c>
       <c r="G4" s="11" t="s">
         <v>13</v>
@@ -1490,7 +1564,7 @@
       </c>
       <c r="F5" s="18">
         <f>F4*C7</f>
-        <v>15.66</v>
+        <v>17.6175</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>13</v>
@@ -1522,7 +1596,7 @@
       </c>
       <c r="F6" s="12">
         <f>(F4+F5)*C9</f>
-        <v>117.44999999999999</v>
+        <v>132.13125000000002</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>13</v>
@@ -1544,7 +1618,7 @@
         <v>9</v>
       </c>
       <c r="C8" s="10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>10</v>
@@ -1568,17 +1642,17 @@
         <v>0.65</v>
       </c>
       <c r="D10" s="11"/>
-      <c r="E10" s="38" t="s">
+      <c r="E10" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="39"/>
-      <c r="G10" s="40"/>
-      <c r="H10" s="50">
+      <c r="F10" s="32"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="37">
         <f>(I5/F6) - 1</f>
-        <v>0.81573588601136215</v>
-      </c>
-      <c r="I10" s="51"/>
-      <c r="J10" s="52"/>
+        <v>0.61398745423232137</v>
+      </c>
+      <c r="I10" s="38"/>
+      <c r="J10" s="39"/>
     </row>
     <row r="11" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B11" s="4" t="s">
@@ -1588,42 +1662,42 @@
         <v>40</v>
       </c>
       <c r="D11" s="6"/>
-      <c r="E11" s="41"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="53"/>
-      <c r="I11" s="54"/>
-      <c r="J11" s="55"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="35"/>
+      <c r="G11" s="36"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="41"/>
+      <c r="J11" s="42"/>
     </row>
     <row r="14" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="15" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B15" s="33" t="s">
+      <c r="B15" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="34"/>
-      <c r="I15" s="34"/>
-      <c r="J15" s="35"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="28"/>
     </row>
     <row r="16" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B16" s="36" t="s">
+      <c r="B16" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="C16" s="37"/>
+      <c r="C16" s="30"/>
       <c r="D16" s="8"/>
-      <c r="E16" s="37" t="s">
+      <c r="E16" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="F16" s="37"/>
+      <c r="F16" s="30"/>
       <c r="G16" s="8"/>
-      <c r="H16" s="37" t="s">
+      <c r="H16" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="I16" s="37"/>
+      <c r="I16" s="30"/>
       <c r="J16" s="9"/>
     </row>
     <row r="17" spans="2:10" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
@@ -1765,17 +1839,17 @@
       <c r="D24" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="E24" s="38" t="s">
+      <c r="E24" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="F24" s="39"/>
-      <c r="G24" s="40"/>
-      <c r="H24" s="44">
+      <c r="F24" s="32"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="43">
         <f>(I18/F19) - 1</f>
         <v>3.7705764438076423</v>
       </c>
-      <c r="I24" s="45"/>
-      <c r="J24" s="46"/>
+      <c r="I24" s="44"/>
+      <c r="J24" s="45"/>
     </row>
     <row r="25" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B25" s="4" t="s">
@@ -1785,220 +1859,220 @@
         <v>1.5</v>
       </c>
       <c r="D25" s="6"/>
-      <c r="E25" s="41"/>
-      <c r="F25" s="42"/>
-      <c r="G25" s="43"/>
-      <c r="H25" s="47"/>
-      <c r="I25" s="48"/>
-      <c r="J25" s="49"/>
+      <c r="E25" s="34"/>
+      <c r="F25" s="35"/>
+      <c r="G25" s="36"/>
+      <c r="H25" s="46"/>
+      <c r="I25" s="47"/>
+      <c r="J25" s="48"/>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B27" s="32" t="e" vm="1">
+      <c r="B27" s="55" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32"/>
-      <c r="H27" s="32"/>
-      <c r="I27" s="32"/>
-      <c r="J27" s="32"/>
+      <c r="C27" s="55"/>
+      <c r="D27" s="55"/>
+      <c r="E27" s="55"/>
+      <c r="F27" s="55"/>
+      <c r="G27" s="55"/>
+      <c r="H27" s="55"/>
+      <c r="I27" s="55"/>
+      <c r="J27" s="55"/>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B28" s="32"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="32"/>
-      <c r="I28" s="32"/>
-      <c r="J28" s="32"/>
+      <c r="B28" s="55"/>
+      <c r="C28" s="55"/>
+      <c r="D28" s="55"/>
+      <c r="E28" s="55"/>
+      <c r="F28" s="55"/>
+      <c r="G28" s="55"/>
+      <c r="H28" s="55"/>
+      <c r="I28" s="55"/>
+      <c r="J28" s="55"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B29" s="32"/>
-      <c r="C29" s="32"/>
-      <c r="D29" s="32"/>
-      <c r="E29" s="32"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="32"/>
-      <c r="H29" s="32"/>
-      <c r="I29" s="32"/>
-      <c r="J29" s="32"/>
+      <c r="B29" s="55"/>
+      <c r="C29" s="55"/>
+      <c r="D29" s="55"/>
+      <c r="E29" s="55"/>
+      <c r="F29" s="55"/>
+      <c r="G29" s="55"/>
+      <c r="H29" s="55"/>
+      <c r="I29" s="55"/>
+      <c r="J29" s="55"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B30" s="32"/>
-      <c r="C30" s="32"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="32"/>
-      <c r="I30" s="32"/>
-      <c r="J30" s="32"/>
+      <c r="B30" s="55"/>
+      <c r="C30" s="55"/>
+      <c r="D30" s="55"/>
+      <c r="E30" s="55"/>
+      <c r="F30" s="55"/>
+      <c r="G30" s="55"/>
+      <c r="H30" s="55"/>
+      <c r="I30" s="55"/>
+      <c r="J30" s="55"/>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B31" s="32"/>
-      <c r="C31" s="32"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="32"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="32"/>
-      <c r="H31" s="32"/>
-      <c r="I31" s="32"/>
-      <c r="J31" s="32"/>
+      <c r="B31" s="55"/>
+      <c r="C31" s="55"/>
+      <c r="D31" s="55"/>
+      <c r="E31" s="55"/>
+      <c r="F31" s="55"/>
+      <c r="G31" s="55"/>
+      <c r="H31" s="55"/>
+      <c r="I31" s="55"/>
+      <c r="J31" s="55"/>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B32" s="32"/>
-      <c r="C32" s="32"/>
-      <c r="D32" s="32"/>
-      <c r="E32" s="32"/>
-      <c r="F32" s="32"/>
-      <c r="G32" s="32"/>
-      <c r="H32" s="32"/>
-      <c r="I32" s="32"/>
-      <c r="J32" s="32"/>
+      <c r="B32" s="55"/>
+      <c r="C32" s="55"/>
+      <c r="D32" s="55"/>
+      <c r="E32" s="55"/>
+      <c r="F32" s="55"/>
+      <c r="G32" s="55"/>
+      <c r="H32" s="55"/>
+      <c r="I32" s="55"/>
+      <c r="J32" s="55"/>
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B33" s="32"/>
-      <c r="C33" s="32"/>
-      <c r="D33" s="32"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
-      <c r="H33" s="32"/>
-      <c r="I33" s="32"/>
-      <c r="J33" s="32"/>
+      <c r="B33" s="55"/>
+      <c r="C33" s="55"/>
+      <c r="D33" s="55"/>
+      <c r="E33" s="55"/>
+      <c r="F33" s="55"/>
+      <c r="G33" s="55"/>
+      <c r="H33" s="55"/>
+      <c r="I33" s="55"/>
+      <c r="J33" s="55"/>
     </row>
     <row r="34" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B34" s="32"/>
-      <c r="C34" s="32"/>
-      <c r="D34" s="32"/>
-      <c r="E34" s="32"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="32"/>
-      <c r="H34" s="32"/>
-      <c r="I34" s="32"/>
-      <c r="J34" s="32"/>
+      <c r="B34" s="55"/>
+      <c r="C34" s="55"/>
+      <c r="D34" s="55"/>
+      <c r="E34" s="55"/>
+      <c r="F34" s="55"/>
+      <c r="G34" s="55"/>
+      <c r="H34" s="55"/>
+      <c r="I34" s="55"/>
+      <c r="J34" s="55"/>
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B35" s="32"/>
-      <c r="C35" s="32"/>
-      <c r="D35" s="32"/>
-      <c r="E35" s="32"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="32"/>
-      <c r="H35" s="32"/>
-      <c r="I35" s="32"/>
-      <c r="J35" s="32"/>
+      <c r="B35" s="55"/>
+      <c r="C35" s="55"/>
+      <c r="D35" s="55"/>
+      <c r="E35" s="55"/>
+      <c r="F35" s="55"/>
+      <c r="G35" s="55"/>
+      <c r="H35" s="55"/>
+      <c r="I35" s="55"/>
+      <c r="J35" s="55"/>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B36" s="32"/>
-      <c r="C36" s="32"/>
-      <c r="D36" s="32"/>
-      <c r="E36" s="32"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="32"/>
-      <c r="H36" s="32"/>
-      <c r="I36" s="32"/>
-      <c r="J36" s="32"/>
+      <c r="B36" s="55"/>
+      <c r="C36" s="55"/>
+      <c r="D36" s="55"/>
+      <c r="E36" s="55"/>
+      <c r="F36" s="55"/>
+      <c r="G36" s="55"/>
+      <c r="H36" s="55"/>
+      <c r="I36" s="55"/>
+      <c r="J36" s="55"/>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B37" s="32"/>
-      <c r="C37" s="32"/>
-      <c r="D37" s="32"/>
-      <c r="E37" s="32"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="32"/>
-      <c r="H37" s="32"/>
-      <c r="I37" s="32"/>
-      <c r="J37" s="32"/>
+      <c r="B37" s="55"/>
+      <c r="C37" s="55"/>
+      <c r="D37" s="55"/>
+      <c r="E37" s="55"/>
+      <c r="F37" s="55"/>
+      <c r="G37" s="55"/>
+      <c r="H37" s="55"/>
+      <c r="I37" s="55"/>
+      <c r="J37" s="55"/>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B38" s="32"/>
-      <c r="C38" s="32"/>
-      <c r="D38" s="32"/>
-      <c r="E38" s="32"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="32"/>
-      <c r="H38" s="32"/>
-      <c r="I38" s="32"/>
-      <c r="J38" s="32"/>
+      <c r="B38" s="55"/>
+      <c r="C38" s="55"/>
+      <c r="D38" s="55"/>
+      <c r="E38" s="55"/>
+      <c r="F38" s="55"/>
+      <c r="G38" s="55"/>
+      <c r="H38" s="55"/>
+      <c r="I38" s="55"/>
+      <c r="J38" s="55"/>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B39" s="32"/>
-      <c r="C39" s="32"/>
-      <c r="D39" s="32"/>
-      <c r="E39" s="32"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="32"/>
-      <c r="H39" s="32"/>
-      <c r="I39" s="32"/>
-      <c r="J39" s="32"/>
+      <c r="B39" s="55"/>
+      <c r="C39" s="55"/>
+      <c r="D39" s="55"/>
+      <c r="E39" s="55"/>
+      <c r="F39" s="55"/>
+      <c r="G39" s="55"/>
+      <c r="H39" s="55"/>
+      <c r="I39" s="55"/>
+      <c r="J39" s="55"/>
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B40" s="32"/>
-      <c r="C40" s="32"/>
-      <c r="D40" s="32"/>
-      <c r="E40" s="32"/>
-      <c r="F40" s="32"/>
-      <c r="G40" s="32"/>
-      <c r="H40" s="32"/>
-      <c r="I40" s="32"/>
-      <c r="J40" s="32"/>
+      <c r="B40" s="55"/>
+      <c r="C40" s="55"/>
+      <c r="D40" s="55"/>
+      <c r="E40" s="55"/>
+      <c r="F40" s="55"/>
+      <c r="G40" s="55"/>
+      <c r="H40" s="55"/>
+      <c r="I40" s="55"/>
+      <c r="J40" s="55"/>
     </row>
     <row r="41" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B41" s="32"/>
-      <c r="C41" s="32"/>
-      <c r="D41" s="32"/>
-      <c r="E41" s="32"/>
-      <c r="F41" s="32"/>
-      <c r="G41" s="32"/>
-      <c r="H41" s="32"/>
-      <c r="I41" s="32"/>
-      <c r="J41" s="32"/>
+      <c r="B41" s="55"/>
+      <c r="C41" s="55"/>
+      <c r="D41" s="55"/>
+      <c r="E41" s="55"/>
+      <c r="F41" s="55"/>
+      <c r="G41" s="55"/>
+      <c r="H41" s="55"/>
+      <c r="I41" s="55"/>
+      <c r="J41" s="55"/>
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="32"/>
-      <c r="H42" s="32"/>
-      <c r="I42" s="32"/>
-      <c r="J42" s="32"/>
+      <c r="B42" s="55"/>
+      <c r="C42" s="55"/>
+      <c r="D42" s="55"/>
+      <c r="E42" s="55"/>
+      <c r="F42" s="55"/>
+      <c r="G42" s="55"/>
+      <c r="H42" s="55"/>
+      <c r="I42" s="55"/>
+      <c r="J42" s="55"/>
     </row>
     <row r="43" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B43" s="32"/>
-      <c r="C43" s="32"/>
-      <c r="D43" s="32"/>
-      <c r="E43" s="32"/>
-      <c r="F43" s="32"/>
-      <c r="G43" s="32"/>
-      <c r="H43" s="32"/>
-      <c r="I43" s="32"/>
-      <c r="J43" s="32"/>
+      <c r="B43" s="55"/>
+      <c r="C43" s="55"/>
+      <c r="D43" s="55"/>
+      <c r="E43" s="55"/>
+      <c r="F43" s="55"/>
+      <c r="G43" s="55"/>
+      <c r="H43" s="55"/>
+      <c r="I43" s="55"/>
+      <c r="J43" s="55"/>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B44" s="32"/>
-      <c r="C44" s="32"/>
-      <c r="D44" s="32"/>
-      <c r="E44" s="32"/>
-      <c r="F44" s="32"/>
-      <c r="G44" s="32"/>
-      <c r="H44" s="32"/>
-      <c r="I44" s="32"/>
-      <c r="J44" s="32"/>
+      <c r="B44" s="55"/>
+      <c r="C44" s="55"/>
+      <c r="D44" s="55"/>
+      <c r="E44" s="55"/>
+      <c r="F44" s="55"/>
+      <c r="G44" s="55"/>
+      <c r="H44" s="55"/>
+      <c r="I44" s="55"/>
+      <c r="J44" s="55"/>
     </row>
     <row r="47" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="48" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B48" s="26" t="s">
+      <c r="B48" s="49" t="s">
         <v>80</v>
       </c>
-      <c r="C48" s="27"/>
-      <c r="D48" s="28"/>
+      <c r="C48" s="50"/>
+      <c r="D48" s="51"/>
       <c r="E48" s="11"/>
       <c r="F48" s="11"/>
       <c r="G48" s="11"/>
@@ -2007,11 +2081,11 @@
       <c r="J48" s="11"/>
     </row>
     <row r="49" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B49" s="29" t="s">
+      <c r="B49" s="52" t="s">
         <v>81</v>
       </c>
-      <c r="C49" s="30"/>
-      <c r="D49" s="31"/>
+      <c r="C49" s="53"/>
+      <c r="D49" s="54"/>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B50" s="2" t="s">
@@ -2062,11 +2136,11 @@
       <c r="D54" s="1"/>
     </row>
     <row r="55" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B55" s="29" t="s">
+      <c r="B55" s="52" t="s">
         <v>85</v>
       </c>
-      <c r="C55" s="30"/>
-      <c r="D55" s="31"/>
+      <c r="C55" s="53"/>
+      <c r="D55" s="54"/>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B56" s="2" t="s">
@@ -2117,11 +2191,11 @@
       <c r="D60" s="1"/>
     </row>
     <row r="61" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B61" s="29" t="s">
+      <c r="B61" s="52" t="s">
         <v>86</v>
       </c>
-      <c r="C61" s="30"/>
-      <c r="D61" s="31"/>
+      <c r="C61" s="53"/>
+      <c r="D61" s="54"/>
     </row>
     <row r="62" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B62" s="2" t="s">
@@ -2229,25 +2303,154 @@
         <v>2</v>
       </c>
     </row>
+    <row r="72" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="73" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B73" s="49" t="s">
+        <v>97</v>
+      </c>
+      <c r="C73" s="50"/>
+      <c r="D73" s="51"/>
+    </row>
+    <row r="74" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B74" s="59" t="s">
+        <v>98</v>
+      </c>
+      <c r="C74" s="60">
+        <f>28*10^6</f>
+        <v>28000000</v>
+      </c>
+      <c r="D74" s="61" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="75" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B75" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C75" s="62">
+        <v>0.28899999999999998</v>
+      </c>
+      <c r="D75" s="15" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="76" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B76" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C76" s="62">
+        <v>0.25</v>
+      </c>
+      <c r="D76" s="15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="77" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B77" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C77" s="62">
+        <v>10.26</v>
+      </c>
+      <c r="D77" s="15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B78" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C78" s="10">
+        <v>2</v>
+      </c>
+      <c r="D78" s="15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="79" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B79" s="2"/>
+      <c r="D79" s="15"/>
+    </row>
+    <row r="80" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B80" s="66" t="s">
+        <v>109</v>
+      </c>
+      <c r="C80" s="3">
+        <f>(PI()*C76^2)/(4)</f>
+        <v>4.9087385212340517E-2</v>
+      </c>
+      <c r="D80" s="64" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="81" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B81" s="66" t="s">
+        <v>110</v>
+      </c>
+      <c r="C81" s="3">
+        <f>C80*C77</f>
+        <v>0.50363657227861369</v>
+      </c>
+      <c r="D81" s="64" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="82" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B82" s="67" t="s">
+        <v>108</v>
+      </c>
+      <c r="C82" s="12">
+        <f>C75*C81</f>
+        <v>0.14555096938851936</v>
+      </c>
+      <c r="D82" s="15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="83" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B83" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C83" s="63">
+        <f>(PI()*POWER(C76,4)) / 64</f>
+        <v>1.9174759848570515E-4</v>
+      </c>
+      <c r="D83" s="64" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="84" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B84" s="68" t="s">
+        <v>107</v>
+      </c>
+      <c r="C84" s="24">
+        <f>(C78*(POWER(C77,3)))/(3*C74*C83)</f>
+        <v>0.13411052373133084</v>
+      </c>
+      <c r="D84" s="65" t="s">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
+    <mergeCell ref="B73:D73"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="B27:J44"/>
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="E24:G25"/>
+    <mergeCell ref="H24:J25"/>
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="H3:I3"/>
     <mergeCell ref="E10:G11"/>
     <mergeCell ref="H10:J11"/>
-    <mergeCell ref="B15:J15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="E24:G25"/>
-    <mergeCell ref="H24:J25"/>
-    <mergeCell ref="B48:D48"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="B61:D61"/>
-    <mergeCell ref="B27:J44"/>
   </mergeCells>
   <conditionalFormatting sqref="H10">
     <cfRule type="colorScale" priority="2">
@@ -2292,17 +2495,17 @@
   <sheetData>
     <row r="1" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="28"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="51"/>
     </row>
     <row r="3" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B3" s="56" t="s">
@@ -2522,17 +2725,17 @@
       <c r="D14" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="38" t="s">
+      <c r="E14" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="F14" s="39"/>
-      <c r="G14" s="39"/>
-      <c r="H14" s="50">
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="37">
         <f>(I5/F9) - 1</f>
         <v>0.44386198487123418</v>
       </c>
-      <c r="I14" s="51"/>
-      <c r="J14" s="52"/>
+      <c r="I14" s="38"/>
+      <c r="J14" s="39"/>
     </row>
     <row r="15" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B15" s="4" t="s">
@@ -2544,23 +2747,23 @@
       <c r="D15" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="41"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="42"/>
-      <c r="H15" s="53"/>
-      <c r="I15" s="54"/>
-      <c r="J15" s="55"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="35"/>
+      <c r="G15" s="35"/>
+      <c r="H15" s="40"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="42"/>
     </row>
     <row r="16" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="17" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="28"/>
+      <c r="C17" s="50"/>
+      <c r="D17" s="50"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="50"/>
+      <c r="G17" s="51"/>
     </row>
     <row r="18" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B18" s="56" t="s">

</xml_diff>

<commit_message>
Minor chages, added FEA
</commit_message>
<xml_diff>
--- a/Analysis/APWCR_Hand_Calculations.xlsx
+++ b/Analysis/APWCR_Hand_Calculations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshu\Documents\UT_Files\Senior_Design_Repos\APWCR_CAD_FILES\Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1308E3C-3F5E-49A6-B419-18DA2A40EE23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{569AA7D8-CDCC-40FC-B821-DCF47FB60FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -432,7 +432,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="167" formatCode="0.000000"/>
+    <numFmt numFmtId="165" formatCode="0.000000"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -804,7 +804,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -831,115 +831,111 @@
     <xf numFmtId="164" fontId="3" fillId="3" borderId="20" xfId="3" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="3" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="3" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Calculation" xfId="3" builtinId="22"/>
@@ -1488,33 +1484,33 @@
   <sheetData>
     <row r="1" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:10" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="28"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
+      <c r="J2" s="41"/>
     </row>
     <row r="3" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="30"/>
+      <c r="C3" s="43"/>
       <c r="D3" s="8"/>
-      <c r="E3" s="30" t="s">
+      <c r="E3" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="30"/>
+      <c r="F3" s="43"/>
       <c r="G3" s="8"/>
-      <c r="H3" s="30" t="s">
+      <c r="H3" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="30"/>
+      <c r="I3" s="43"/>
       <c r="J3" s="9"/>
     </row>
     <row r="4" spans="2:10" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
@@ -1642,17 +1638,17 @@
         <v>0.65</v>
       </c>
       <c r="D10" s="11"/>
-      <c r="E10" s="31" t="s">
+      <c r="E10" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="32"/>
-      <c r="G10" s="33"/>
-      <c r="H10" s="37">
+      <c r="F10" s="45"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="56">
         <f>(I5/F6) - 1</f>
         <v>0.61398745423232137</v>
       </c>
-      <c r="I10" s="38"/>
-      <c r="J10" s="39"/>
+      <c r="I10" s="57"/>
+      <c r="J10" s="58"/>
     </row>
     <row r="11" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B11" s="4" t="s">
@@ -1662,42 +1658,42 @@
         <v>40</v>
       </c>
       <c r="D11" s="6"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="36"/>
-      <c r="H11" s="40"/>
-      <c r="I11" s="41"/>
-      <c r="J11" s="42"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="48"/>
+      <c r="G11" s="49"/>
+      <c r="H11" s="59"/>
+      <c r="I11" s="60"/>
+      <c r="J11" s="61"/>
     </row>
     <row r="14" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="15" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="39" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="28"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="40"/>
+      <c r="G15" s="40"/>
+      <c r="H15" s="40"/>
+      <c r="I15" s="40"/>
+      <c r="J15" s="41"/>
     </row>
     <row r="16" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B16" s="29" t="s">
+      <c r="B16" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C16" s="30"/>
+      <c r="C16" s="43"/>
       <c r="D16" s="8"/>
-      <c r="E16" s="30" t="s">
+      <c r="E16" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="F16" s="30"/>
+      <c r="F16" s="43"/>
       <c r="G16" s="8"/>
-      <c r="H16" s="30" t="s">
+      <c r="H16" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="I16" s="30"/>
+      <c r="I16" s="43"/>
       <c r="J16" s="9"/>
     </row>
     <row r="17" spans="2:10" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
@@ -1839,17 +1835,17 @@
       <c r="D24" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="E24" s="31" t="s">
+      <c r="E24" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="F24" s="32"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="43">
+      <c r="F24" s="45"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="50">
         <f>(I18/F19) - 1</f>
         <v>3.7705764438076423</v>
       </c>
-      <c r="I24" s="44"/>
-      <c r="J24" s="45"/>
+      <c r="I24" s="51"/>
+      <c r="J24" s="52"/>
     </row>
     <row r="25" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B25" s="4" t="s">
@@ -1859,220 +1855,220 @@
         <v>1.5</v>
       </c>
       <c r="D25" s="6"/>
-      <c r="E25" s="34"/>
-      <c r="F25" s="35"/>
-      <c r="G25" s="36"/>
-      <c r="H25" s="46"/>
-      <c r="I25" s="47"/>
-      <c r="J25" s="48"/>
+      <c r="E25" s="47"/>
+      <c r="F25" s="48"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="53"/>
+      <c r="I25" s="54"/>
+      <c r="J25" s="55"/>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B27" s="55" t="e" vm="1">
+      <c r="B27" s="38" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C27" s="55"/>
-      <c r="D27" s="55"/>
-      <c r="E27" s="55"/>
-      <c r="F27" s="55"/>
-      <c r="G27" s="55"/>
-      <c r="H27" s="55"/>
-      <c r="I27" s="55"/>
-      <c r="J27" s="55"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="38"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="38"/>
+      <c r="I27" s="38"/>
+      <c r="J27" s="38"/>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B28" s="55"/>
-      <c r="C28" s="55"/>
-      <c r="D28" s="55"/>
-      <c r="E28" s="55"/>
-      <c r="F28" s="55"/>
-      <c r="G28" s="55"/>
-      <c r="H28" s="55"/>
-      <c r="I28" s="55"/>
-      <c r="J28" s="55"/>
+      <c r="B28" s="38"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="38"/>
+      <c r="J28" s="38"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B29" s="55"/>
-      <c r="C29" s="55"/>
-      <c r="D29" s="55"/>
-      <c r="E29" s="55"/>
-      <c r="F29" s="55"/>
-      <c r="G29" s="55"/>
-      <c r="H29" s="55"/>
-      <c r="I29" s="55"/>
-      <c r="J29" s="55"/>
+      <c r="B29" s="38"/>
+      <c r="C29" s="38"/>
+      <c r="D29" s="38"/>
+      <c r="E29" s="38"/>
+      <c r="F29" s="38"/>
+      <c r="G29" s="38"/>
+      <c r="H29" s="38"/>
+      <c r="I29" s="38"/>
+      <c r="J29" s="38"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B30" s="55"/>
-      <c r="C30" s="55"/>
-      <c r="D30" s="55"/>
-      <c r="E30" s="55"/>
-      <c r="F30" s="55"/>
-      <c r="G30" s="55"/>
-      <c r="H30" s="55"/>
-      <c r="I30" s="55"/>
-      <c r="J30" s="55"/>
+      <c r="B30" s="38"/>
+      <c r="C30" s="38"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="38"/>
+      <c r="F30" s="38"/>
+      <c r="G30" s="38"/>
+      <c r="H30" s="38"/>
+      <c r="I30" s="38"/>
+      <c r="J30" s="38"/>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B31" s="55"/>
-      <c r="C31" s="55"/>
-      <c r="D31" s="55"/>
-      <c r="E31" s="55"/>
-      <c r="F31" s="55"/>
-      <c r="G31" s="55"/>
-      <c r="H31" s="55"/>
-      <c r="I31" s="55"/>
-      <c r="J31" s="55"/>
+      <c r="B31" s="38"/>
+      <c r="C31" s="38"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="38"/>
+      <c r="F31" s="38"/>
+      <c r="G31" s="38"/>
+      <c r="H31" s="38"/>
+      <c r="I31" s="38"/>
+      <c r="J31" s="38"/>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B32" s="55"/>
-      <c r="C32" s="55"/>
-      <c r="D32" s="55"/>
-      <c r="E32" s="55"/>
-      <c r="F32" s="55"/>
-      <c r="G32" s="55"/>
-      <c r="H32" s="55"/>
-      <c r="I32" s="55"/>
-      <c r="J32" s="55"/>
+      <c r="B32" s="38"/>
+      <c r="C32" s="38"/>
+      <c r="D32" s="38"/>
+      <c r="E32" s="38"/>
+      <c r="F32" s="38"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="38"/>
+      <c r="I32" s="38"/>
+      <c r="J32" s="38"/>
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B33" s="55"/>
-      <c r="C33" s="55"/>
-      <c r="D33" s="55"/>
-      <c r="E33" s="55"/>
-      <c r="F33" s="55"/>
-      <c r="G33" s="55"/>
-      <c r="H33" s="55"/>
-      <c r="I33" s="55"/>
-      <c r="J33" s="55"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="38"/>
+      <c r="I33" s="38"/>
+      <c r="J33" s="38"/>
     </row>
     <row r="34" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B34" s="55"/>
-      <c r="C34" s="55"/>
-      <c r="D34" s="55"/>
-      <c r="E34" s="55"/>
-      <c r="F34" s="55"/>
-      <c r="G34" s="55"/>
-      <c r="H34" s="55"/>
-      <c r="I34" s="55"/>
-      <c r="J34" s="55"/>
+      <c r="B34" s="38"/>
+      <c r="C34" s="38"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="38"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="38"/>
+      <c r="I34" s="38"/>
+      <c r="J34" s="38"/>
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B35" s="55"/>
-      <c r="C35" s="55"/>
-      <c r="D35" s="55"/>
-      <c r="E35" s="55"/>
-      <c r="F35" s="55"/>
-      <c r="G35" s="55"/>
-      <c r="H35" s="55"/>
-      <c r="I35" s="55"/>
-      <c r="J35" s="55"/>
+      <c r="B35" s="38"/>
+      <c r="C35" s="38"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="38"/>
+      <c r="F35" s="38"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="38"/>
+      <c r="I35" s="38"/>
+      <c r="J35" s="38"/>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B36" s="55"/>
-      <c r="C36" s="55"/>
-      <c r="D36" s="55"/>
-      <c r="E36" s="55"/>
-      <c r="F36" s="55"/>
-      <c r="G36" s="55"/>
-      <c r="H36" s="55"/>
-      <c r="I36" s="55"/>
-      <c r="J36" s="55"/>
+      <c r="B36" s="38"/>
+      <c r="C36" s="38"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="38"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="38"/>
+      <c r="I36" s="38"/>
+      <c r="J36" s="38"/>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B37" s="55"/>
-      <c r="C37" s="55"/>
-      <c r="D37" s="55"/>
-      <c r="E37" s="55"/>
-      <c r="F37" s="55"/>
-      <c r="G37" s="55"/>
-      <c r="H37" s="55"/>
-      <c r="I37" s="55"/>
-      <c r="J37" s="55"/>
+      <c r="B37" s="38"/>
+      <c r="C37" s="38"/>
+      <c r="D37" s="38"/>
+      <c r="E37" s="38"/>
+      <c r="F37" s="38"/>
+      <c r="G37" s="38"/>
+      <c r="H37" s="38"/>
+      <c r="I37" s="38"/>
+      <c r="J37" s="38"/>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B38" s="55"/>
-      <c r="C38" s="55"/>
-      <c r="D38" s="55"/>
-      <c r="E38" s="55"/>
-      <c r="F38" s="55"/>
-      <c r="G38" s="55"/>
-      <c r="H38" s="55"/>
-      <c r="I38" s="55"/>
-      <c r="J38" s="55"/>
+      <c r="B38" s="38"/>
+      <c r="C38" s="38"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="38"/>
+      <c r="G38" s="38"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="38"/>
+      <c r="J38" s="38"/>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B39" s="55"/>
-      <c r="C39" s="55"/>
-      <c r="D39" s="55"/>
-      <c r="E39" s="55"/>
-      <c r="F39" s="55"/>
-      <c r="G39" s="55"/>
-      <c r="H39" s="55"/>
-      <c r="I39" s="55"/>
-      <c r="J39" s="55"/>
+      <c r="B39" s="38"/>
+      <c r="C39" s="38"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="38"/>
+      <c r="F39" s="38"/>
+      <c r="G39" s="38"/>
+      <c r="H39" s="38"/>
+      <c r="I39" s="38"/>
+      <c r="J39" s="38"/>
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B40" s="55"/>
-      <c r="C40" s="55"/>
-      <c r="D40" s="55"/>
-      <c r="E40" s="55"/>
-      <c r="F40" s="55"/>
-      <c r="G40" s="55"/>
-      <c r="H40" s="55"/>
-      <c r="I40" s="55"/>
-      <c r="J40" s="55"/>
+      <c r="B40" s="38"/>
+      <c r="C40" s="38"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="38"/>
+      <c r="F40" s="38"/>
+      <c r="G40" s="38"/>
+      <c r="H40" s="38"/>
+      <c r="I40" s="38"/>
+      <c r="J40" s="38"/>
     </row>
     <row r="41" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B41" s="55"/>
-      <c r="C41" s="55"/>
-      <c r="D41" s="55"/>
-      <c r="E41" s="55"/>
-      <c r="F41" s="55"/>
-      <c r="G41" s="55"/>
-      <c r="H41" s="55"/>
-      <c r="I41" s="55"/>
-      <c r="J41" s="55"/>
+      <c r="B41" s="38"/>
+      <c r="C41" s="38"/>
+      <c r="D41" s="38"/>
+      <c r="E41" s="38"/>
+      <c r="F41" s="38"/>
+      <c r="G41" s="38"/>
+      <c r="H41" s="38"/>
+      <c r="I41" s="38"/>
+      <c r="J41" s="38"/>
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B42" s="55"/>
-      <c r="C42" s="55"/>
-      <c r="D42" s="55"/>
-      <c r="E42" s="55"/>
-      <c r="F42" s="55"/>
-      <c r="G42" s="55"/>
-      <c r="H42" s="55"/>
-      <c r="I42" s="55"/>
-      <c r="J42" s="55"/>
+      <c r="B42" s="38"/>
+      <c r="C42" s="38"/>
+      <c r="D42" s="38"/>
+      <c r="E42" s="38"/>
+      <c r="F42" s="38"/>
+      <c r="G42" s="38"/>
+      <c r="H42" s="38"/>
+      <c r="I42" s="38"/>
+      <c r="J42" s="38"/>
     </row>
     <row r="43" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B43" s="55"/>
-      <c r="C43" s="55"/>
-      <c r="D43" s="55"/>
-      <c r="E43" s="55"/>
-      <c r="F43" s="55"/>
-      <c r="G43" s="55"/>
-      <c r="H43" s="55"/>
-      <c r="I43" s="55"/>
-      <c r="J43" s="55"/>
+      <c r="B43" s="38"/>
+      <c r="C43" s="38"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38"/>
+      <c r="F43" s="38"/>
+      <c r="G43" s="38"/>
+      <c r="H43" s="38"/>
+      <c r="I43" s="38"/>
+      <c r="J43" s="38"/>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B44" s="55"/>
-      <c r="C44" s="55"/>
-      <c r="D44" s="55"/>
-      <c r="E44" s="55"/>
-      <c r="F44" s="55"/>
-      <c r="G44" s="55"/>
-      <c r="H44" s="55"/>
-      <c r="I44" s="55"/>
-      <c r="J44" s="55"/>
+      <c r="B44" s="38"/>
+      <c r="C44" s="38"/>
+      <c r="D44" s="38"/>
+      <c r="E44" s="38"/>
+      <c r="F44" s="38"/>
+      <c r="G44" s="38"/>
+      <c r="H44" s="38"/>
+      <c r="I44" s="38"/>
+      <c r="J44" s="38"/>
     </row>
     <row r="47" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="48" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B48" s="49" t="s">
+      <c r="B48" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="C48" s="50"/>
-      <c r="D48" s="51"/>
+      <c r="C48" s="33"/>
+      <c r="D48" s="34"/>
       <c r="E48" s="11"/>
       <c r="F48" s="11"/>
       <c r="G48" s="11"/>
@@ -2081,11 +2077,11 @@
       <c r="J48" s="11"/>
     </row>
     <row r="49" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B49" s="52" t="s">
+      <c r="B49" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="C49" s="53"/>
-      <c r="D49" s="54"/>
+      <c r="C49" s="36"/>
+      <c r="D49" s="37"/>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B50" s="2" t="s">
@@ -2136,11 +2132,11 @@
       <c r="D54" s="1"/>
     </row>
     <row r="55" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B55" s="52" t="s">
+      <c r="B55" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="C55" s="53"/>
-      <c r="D55" s="54"/>
+      <c r="C55" s="36"/>
+      <c r="D55" s="37"/>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B56" s="2" t="s">
@@ -2191,11 +2187,11 @@
       <c r="D60" s="1"/>
     </row>
     <row r="61" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B61" s="52" t="s">
+      <c r="B61" s="35" t="s">
         <v>86</v>
       </c>
-      <c r="C61" s="53"/>
-      <c r="D61" s="54"/>
+      <c r="C61" s="36"/>
+      <c r="D61" s="37"/>
     </row>
     <row r="62" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B62" s="2" t="s">
@@ -2305,21 +2301,21 @@
     </row>
     <row r="72" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="73" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B73" s="49" t="s">
+      <c r="B73" s="32" t="s">
         <v>97</v>
       </c>
-      <c r="C73" s="50"/>
-      <c r="D73" s="51"/>
+      <c r="C73" s="33"/>
+      <c r="D73" s="34"/>
     </row>
     <row r="74" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B74" s="59" t="s">
+      <c r="B74" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="C74" s="60">
+      <c r="C74" s="27">
         <f>28*10^6</f>
         <v>28000000</v>
       </c>
-      <c r="D74" s="61" t="s">
+      <c r="D74" s="28" t="s">
         <v>100</v>
       </c>
     </row>
@@ -2327,7 +2323,7 @@
       <c r="B75" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C75" s="62">
+      <c r="C75" s="10">
         <v>0.28899999999999998</v>
       </c>
       <c r="D75" s="15" t="s">
@@ -2338,7 +2334,7 @@
       <c r="B76" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C76" s="62">
+      <c r="C76" s="10">
         <v>0.25</v>
       </c>
       <c r="D76" s="15" t="s">
@@ -2349,7 +2345,7 @@
       <c r="B77" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C77" s="62">
+      <c r="C77" s="10">
         <v>10.26</v>
       </c>
       <c r="D77" s="15" t="s">
@@ -2361,7 +2357,7 @@
         <v>106</v>
       </c>
       <c r="C78" s="10">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D78" s="15" t="s">
         <v>32</v>
@@ -2372,31 +2368,31 @@
       <c r="D79" s="15"/>
     </row>
     <row r="80" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B80" s="66" t="s">
+      <c r="B80" s="2" t="s">
         <v>109</v>
       </c>
       <c r="C80" s="3">
         <f>(PI()*C76^2)/(4)</f>
         <v>4.9087385212340517E-2</v>
       </c>
-      <c r="D80" s="64" t="s">
+      <c r="D80" s="15" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="81" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B81" s="66" t="s">
+      <c r="B81" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C81" s="3">
         <f>C80*C77</f>
         <v>0.50363657227861369</v>
       </c>
-      <c r="D81" s="64" t="s">
+      <c r="D81" s="15" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B82" s="67" t="s">
+      <c r="B82" s="30" t="s">
         <v>108</v>
       </c>
       <c r="C82" s="12">
@@ -2411,33 +2407,34 @@
       <c r="B83" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C83" s="63">
+      <c r="C83" s="29">
         <f>(PI()*POWER(C76,4)) / 64</f>
         <v>1.9174759848570515E-4</v>
       </c>
-      <c r="D83" s="64" t="s">
+      <c r="D83" s="15" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="84" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B84" s="68" t="s">
+      <c r="B84" s="31" t="s">
         <v>107</v>
       </c>
       <c r="C84" s="24">
         <f>(C78*(POWER(C77,3)))/(3*C74*C83)</f>
-        <v>0.13411052373133084</v>
-      </c>
-      <c r="D84" s="65" t="s">
+        <v>0.10058289279849812</v>
+      </c>
+      <c r="D84" s="25" t="s">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B73:D73"/>
-    <mergeCell ref="B48:D48"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="E10:G11"/>
+    <mergeCell ref="H10:J11"/>
     <mergeCell ref="B27:J44"/>
     <mergeCell ref="B15:J15"/>
     <mergeCell ref="B16:C16"/>
@@ -2445,12 +2442,11 @@
     <mergeCell ref="H16:I16"/>
     <mergeCell ref="E24:G25"/>
     <mergeCell ref="H24:J25"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="E10:G11"/>
-    <mergeCell ref="H10:J11"/>
+    <mergeCell ref="B73:D73"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B61:D61"/>
   </mergeCells>
   <conditionalFormatting sqref="H10">
     <cfRule type="colorScale" priority="2">
@@ -2495,33 +2491,33 @@
   <sheetData>
     <row r="1" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="49" t="s">
+      <c r="B2" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
-      <c r="I2" s="50"/>
-      <c r="J2" s="51"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="34"/>
     </row>
     <row r="3" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="56" t="s">
+      <c r="B3" s="62" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="57"/>
+      <c r="C3" s="63"/>
       <c r="D3" s="8"/>
-      <c r="E3" s="56" t="s">
+      <c r="E3" s="62" t="s">
         <v>44</v>
       </c>
-      <c r="F3" s="57"/>
+      <c r="F3" s="63"/>
       <c r="G3" s="8"/>
-      <c r="H3" s="56" t="s">
+      <c r="H3" s="62" t="s">
         <v>45</v>
       </c>
-      <c r="I3" s="57"/>
+      <c r="I3" s="63"/>
       <c r="J3" s="9"/>
     </row>
     <row r="4" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -2725,17 +2721,17 @@
       <c r="D14" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="31" t="s">
+      <c r="E14" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="F14" s="32"/>
-      <c r="G14" s="32"/>
-      <c r="H14" s="37">
+      <c r="F14" s="45"/>
+      <c r="G14" s="45"/>
+      <c r="H14" s="56">
         <f>(I5/F9) - 1</f>
         <v>0.44386198487123418</v>
       </c>
-      <c r="I14" s="38"/>
-      <c r="J14" s="39"/>
+      <c r="I14" s="57"/>
+      <c r="J14" s="58"/>
     </row>
     <row r="15" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B15" s="4" t="s">
@@ -2747,34 +2743,34 @@
       <c r="D15" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="34"/>
-      <c r="F15" s="35"/>
-      <c r="G15" s="35"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="41"/>
-      <c r="J15" s="42"/>
+      <c r="E15" s="47"/>
+      <c r="F15" s="48"/>
+      <c r="G15" s="48"/>
+      <c r="H15" s="59"/>
+      <c r="I15" s="60"/>
+      <c r="J15" s="61"/>
     </row>
     <row r="16" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="17" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B17" s="49" t="s">
+      <c r="B17" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="50"/>
-      <c r="D17" s="50"/>
-      <c r="E17" s="50"/>
-      <c r="F17" s="50"/>
-      <c r="G17" s="51"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="34"/>
     </row>
     <row r="18" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B18" s="56" t="s">
+      <c r="B18" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="C18" s="57"/>
-      <c r="E18" s="56" t="s">
+      <c r="C18" s="63"/>
+      <c r="E18" s="62" t="s">
         <v>58</v>
       </c>
-      <c r="F18" s="58"/>
-      <c r="G18" s="57"/>
+      <c r="F18" s="64"/>
+      <c r="G18" s="63"/>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.45">
       <c r="B19" s="2" t="s">

</xml_diff>